<commit_message>
Added control authority scheme, bit masks for flags, extra frame space for gripper,enc reset etc. Updated Frame info.txt
</commit_message>
<xml_diff>
--- a/Thermo CRS F3 Controller.xlsx
+++ b/Thermo CRS F3 Controller.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="51">
   <si>
     <t>Rx Slave</t>
   </si>
@@ -97,6 +97,87 @@
   </si>
   <si>
     <t>Umbilical Connecor pin assignments</t>
+  </si>
+  <si>
+    <t>Waist</t>
+  </si>
+  <si>
+    <t>Shoulder</t>
+  </si>
+  <si>
+    <t>Elbow</t>
+  </si>
+  <si>
+    <t>Wrist rotate</t>
+  </si>
+  <si>
+    <t>Wrist pitch</t>
+  </si>
+  <si>
+    <t>Tool roll</t>
+  </si>
+  <si>
+    <t>Axis</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>0x10</t>
+  </si>
+  <si>
+    <t>0x08</t>
+  </si>
+  <si>
+    <t>0x11</t>
+  </si>
+  <si>
+    <t>0x09</t>
+  </si>
+  <si>
+    <t>0x12</t>
+  </si>
+  <si>
+    <t>0x0A</t>
+  </si>
+  <si>
+    <t>Node ID</t>
+  </si>
+  <si>
+    <t>Motor RPM</t>
+  </si>
+  <si>
+    <t>100% speed</t>
+  </si>
+  <si>
+    <t>Reduction</t>
+  </si>
+  <si>
+    <t>max. °/s</t>
+  </si>
+  <si>
+    <t>Acceleration</t>
+  </si>
+  <si>
+    <t>Default °/s²</t>
+  </si>
+  <si>
+    <t>Max °/s²</t>
+  </si>
+  <si>
+    <t>Resolution °</t>
+  </si>
+  <si>
+    <t>Pulses/</t>
+  </si>
+  <si>
+    <t>+90°</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 1:X Gear </t>
+  </si>
+  <si>
+    <t>+1°</t>
   </si>
 </sst>
 </file>
@@ -202,7 +283,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -217,6 +298,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -587,8 +674,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="13217620" y="470648"/>
-          <a:ext cx="2179263" cy="451318"/>
+          <a:off x="12837813" y="470648"/>
+          <a:ext cx="1907180" cy="451318"/>
           <a:chOff x="13077825" y="2600325"/>
           <a:chExt cx="3667125" cy="971550"/>
         </a:xfrm>
@@ -896,8 +983,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="13271683" y="1961031"/>
-          <a:ext cx="2270875" cy="464486"/>
+          <a:off x="12834726" y="1961031"/>
+          <a:ext cx="2055942" cy="464486"/>
           <a:chOff x="16992600" y="962025"/>
           <a:chExt cx="3667125" cy="981075"/>
         </a:xfrm>
@@ -1367,8 +1454,8 @@
       <xdr:rowOff>96481</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>17</xdr:col>
-      <xdr:colOff>340734</xdr:colOff>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>108821</xdr:colOff>
       <xdr:row>7</xdr:row>
       <xdr:rowOff>190498</xdr:rowOff>
     </xdr:to>
@@ -1405,8 +1492,8 @@
       <xdr:rowOff>131885</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>17</xdr:col>
-      <xdr:colOff>339625</xdr:colOff>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>107712</xdr:colOff>
       <xdr:row>16</xdr:row>
       <xdr:rowOff>35402</xdr:rowOff>
     </xdr:to>
@@ -1905,8 +1992,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="19117235" y="1322291"/>
-          <a:ext cx="4612341" cy="2482444"/>
+          <a:off x="18390801" y="1322291"/>
+          <a:ext cx="4631830" cy="2482444"/>
           <a:chOff x="11710147" y="8751794"/>
           <a:chExt cx="4612341" cy="2482444"/>
         </a:xfrm>
@@ -2886,7 +2973,7 @@
       <xdr:grpSpPr>
         <a:xfrm>
           <a:off x="888066" y="293177"/>
-          <a:ext cx="8238273" cy="12622839"/>
+          <a:ext cx="8248991" cy="12622839"/>
           <a:chOff x="888066" y="293177"/>
           <a:chExt cx="8238273" cy="12622839"/>
         </a:xfrm>
@@ -3489,6 +3576,158 @@
         </xdr:cxnSp>
       </xdr:grpSp>
     </xdr:grpSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>571501</xdr:colOff>
+      <xdr:row>56</xdr:row>
+      <xdr:rowOff>52389</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>293557</xdr:colOff>
+      <xdr:row>79</xdr:row>
+      <xdr:rowOff>95251</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Grafik 2"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="10882314" y="10720389"/>
+          <a:ext cx="4393448" cy="4424362"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>9525</xdr:colOff>
+      <xdr:row>56</xdr:row>
+      <xdr:rowOff>52388</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>495850</xdr:colOff>
+      <xdr:row>81</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Grafik 4"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="15278100" y="10720388"/>
+          <a:ext cx="2697781" cy="4738687"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>304244</xdr:colOff>
+      <xdr:row>79</xdr:row>
+      <xdr:rowOff>66674</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>203751</xdr:colOff>
+      <xdr:row>119</xdr:row>
+      <xdr:rowOff>5536</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Grafik 5"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9857819" y="15116174"/>
+          <a:ext cx="8306355" cy="7558862"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>278603</xdr:colOff>
+      <xdr:row>56</xdr:row>
+      <xdr:rowOff>32600</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>33</xdr:col>
+      <xdr:colOff>195715</xdr:colOff>
+      <xdr:row>86</xdr:row>
+      <xdr:rowOff>112060</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="Grafik 6"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="17827015" y="10700600"/>
+          <a:ext cx="5430406" cy="5794460"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -10741,6 +10980,10 @@
   <cols>
     <col min="7" max="9" width="9.28515625" customWidth="1"/>
     <col min="10" max="10" width="12.5703125" customWidth="1"/>
+    <col min="17" max="17" width="5.7109375" style="9" customWidth="1"/>
+    <col min="18" max="18" width="9.140625" customWidth="1"/>
+    <col min="20" max="20" width="9.42578125" customWidth="1"/>
+    <col min="22" max="22" width="10.28515625" customWidth="1"/>
     <col min="28" max="32" width="7.42578125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -10910,12 +11153,311 @@
         <v>10</v>
       </c>
     </row>
+    <row r="38" spans="16:27" x14ac:dyDescent="0.25">
+      <c r="S38" t="s">
+        <v>39</v>
+      </c>
+      <c r="T38" t="s">
+        <v>49</v>
+      </c>
+      <c r="V38" s="15" t="s">
+        <v>43</v>
+      </c>
+      <c r="W38" s="15"/>
+      <c r="Y38" t="s">
+        <v>47</v>
+      </c>
+      <c r="Z38" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="39" spans="16:27" x14ac:dyDescent="0.25">
+      <c r="P39" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q39" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="R39" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="S39" t="s">
+        <v>40</v>
+      </c>
+      <c r="T39" t="s">
+        <v>41</v>
+      </c>
+      <c r="U39" t="s">
+        <v>42</v>
+      </c>
+      <c r="V39" t="s">
+        <v>44</v>
+      </c>
+      <c r="W39" t="s">
+        <v>45</v>
+      </c>
+      <c r="X39" t="s">
+        <v>46</v>
+      </c>
+      <c r="Y39" s="14" t="s">
+        <v>48</v>
+      </c>
+      <c r="Z39" s="14" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="40" spans="16:27" x14ac:dyDescent="0.25">
+      <c r="R40" s="9"/>
+    </row>
+    <row r="41" spans="16:27" x14ac:dyDescent="0.25">
+      <c r="P41" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q41" s="9">
+        <v>1</v>
+      </c>
+      <c r="R41" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="S41" s="9">
+        <v>4000</v>
+      </c>
+      <c r="T41" s="13">
+        <v>100</v>
+      </c>
+      <c r="U41" s="13">
+        <v>240</v>
+      </c>
+      <c r="V41" s="9">
+        <v>879</v>
+      </c>
+      <c r="W41" s="9">
+        <v>1757</v>
+      </c>
+      <c r="X41" s="9">
+        <v>1.8E-3</v>
+      </c>
+      <c r="Y41" s="9">
+        <v>-51200</v>
+      </c>
+      <c r="Z41">
+        <f>Y41/90</f>
+        <v>-568.88888888888891</v>
+      </c>
+      <c r="AA41">
+        <f>1/Z41</f>
+        <v>-1.7578124999999998E-3</v>
+      </c>
+    </row>
+    <row r="42" spans="16:27" x14ac:dyDescent="0.25">
+      <c r="P42" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q42" s="9">
+        <v>2</v>
+      </c>
+      <c r="R42" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="S42" s="9">
+        <v>4000</v>
+      </c>
+      <c r="T42" s="13">
+        <v>100</v>
+      </c>
+      <c r="U42" s="13">
+        <v>210</v>
+      </c>
+      <c r="V42" s="9">
+        <v>879</v>
+      </c>
+      <c r="W42" s="9">
+        <v>1757</v>
+      </c>
+      <c r="X42" s="9">
+        <v>1.8E-3</v>
+      </c>
+      <c r="Y42" s="9">
+        <v>51200</v>
+      </c>
+      <c r="Z42">
+        <f t="shared" ref="Z42:Z46" si="0">Y42/90</f>
+        <v>568.88888888888891</v>
+      </c>
+      <c r="AA42">
+        <f t="shared" ref="AA42:AA46" si="1">1/Z42</f>
+        <v>1.7578124999999998E-3</v>
+      </c>
+    </row>
+    <row r="43" spans="16:27" x14ac:dyDescent="0.25">
+      <c r="P43" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q43" s="9">
+        <v>3</v>
+      </c>
+      <c r="R43" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="S43" s="9">
+        <v>4000</v>
+      </c>
+      <c r="T43" s="13">
+        <v>100</v>
+      </c>
+      <c r="U43" s="13">
+        <v>240</v>
+      </c>
+      <c r="V43" s="9">
+        <v>879</v>
+      </c>
+      <c r="W43" s="9">
+        <v>2636</v>
+      </c>
+      <c r="X43" s="9">
+        <v>1.8E-3</v>
+      </c>
+      <c r="Y43" s="9">
+        <v>51200</v>
+      </c>
+      <c r="Z43">
+        <f t="shared" si="0"/>
+        <v>568.88888888888891</v>
+      </c>
+      <c r="AA43">
+        <f t="shared" si="1"/>
+        <v>1.7578124999999998E-3</v>
+      </c>
+    </row>
+    <row r="44" spans="16:27" x14ac:dyDescent="0.25">
+      <c r="P44" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q44" s="9">
+        <v>4</v>
+      </c>
+      <c r="R44" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="S44" s="9">
+        <v>5000</v>
+      </c>
+      <c r="T44" s="13">
+        <v>80</v>
+      </c>
+      <c r="U44" s="13">
+        <v>375</v>
+      </c>
+      <c r="V44" s="9">
+        <v>1098</v>
+      </c>
+      <c r="W44" s="9">
+        <v>3295</v>
+      </c>
+      <c r="X44" s="9">
+        <v>2.2000000000000001E-3</v>
+      </c>
+      <c r="Y44" s="9">
+        <v>-40960</v>
+      </c>
+      <c r="Z44">
+        <f t="shared" si="0"/>
+        <v>-455.11111111111109</v>
+      </c>
+      <c r="AA44">
+        <f t="shared" si="1"/>
+        <v>-2.197265625E-3</v>
+      </c>
+    </row>
+    <row r="45" spans="16:27" x14ac:dyDescent="0.25">
+      <c r="P45" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q45" s="9">
+        <v>5</v>
+      </c>
+      <c r="R45" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="S45" s="9">
+        <v>4000</v>
+      </c>
+      <c r="T45" s="13">
+        <v>80</v>
+      </c>
+      <c r="U45" s="13">
+        <v>300</v>
+      </c>
+      <c r="V45" s="9">
+        <v>1098</v>
+      </c>
+      <c r="W45" s="9">
+        <v>3295</v>
+      </c>
+      <c r="X45" s="9">
+        <v>2.2000000000000001E-3</v>
+      </c>
+      <c r="Y45" s="9">
+        <v>40960</v>
+      </c>
+      <c r="Z45">
+        <f t="shared" si="0"/>
+        <v>455.11111111111109</v>
+      </c>
+      <c r="AA45">
+        <f t="shared" si="1"/>
+        <v>2.197265625E-3</v>
+      </c>
+    </row>
+    <row r="46" spans="16:27" x14ac:dyDescent="0.25">
+      <c r="P46" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q46" s="9">
+        <v>6</v>
+      </c>
+      <c r="R46" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="S46" s="9">
+        <v>5000</v>
+      </c>
+      <c r="T46" s="13">
+        <v>80</v>
+      </c>
+      <c r="U46" s="13">
+        <v>375</v>
+      </c>
+      <c r="V46" s="9">
+        <v>1098</v>
+      </c>
+      <c r="W46" s="9">
+        <v>3295</v>
+      </c>
+      <c r="X46" s="9">
+        <v>2.2000000000000001E-3</v>
+      </c>
+      <c r="Y46" s="9">
+        <v>-40960</v>
+      </c>
+      <c r="Z46">
+        <f t="shared" si="0"/>
+        <v>-455.11111111111109</v>
+      </c>
+      <c r="AA46">
+        <f t="shared" si="1"/>
+        <v>-2.197265625E-3</v>
+      </c>
+    </row>
     <row r="75" spans="8:8" x14ac:dyDescent="0.25">
       <c r="H75" t="s">
         <v>22</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="V38:W38"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
@@ -10927,9 +11469,19 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1"/>
+  <dimension ref="H60:H62"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <sheetData>
+    <row r="60" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H60" s="12"/>
+    </row>
+    <row r="61" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H61" s="12"/>
+    </row>
+    <row r="62" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H62" s="12"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="68" orientation="landscape" r:id="rId1"/>
   <drawing r:id="rId2"/>

</xml_diff>

<commit_message>
added inverse kinematics with analytic solver as well as forward kinematics. Both uitilizing modified DH-Parameters and solving with respect to the mechanical coupling of j2 & j3
</commit_message>
<xml_diff>
--- a/Thermo CRS F3 Controller.xlsx
+++ b/Thermo CRS F3 Controller.xlsx
@@ -1993,7 +1993,7 @@
       <xdr:grpSpPr>
         <a:xfrm>
           <a:off x="18390801" y="1322291"/>
-          <a:ext cx="4631830" cy="2482444"/>
+          <a:ext cx="4930004" cy="2482444"/>
           <a:chOff x="11710147" y="8751794"/>
           <a:chExt cx="4612341" cy="2482444"/>
         </a:xfrm>
@@ -3700,8 +3700,8 @@
       <xdr:rowOff>32600</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>33</xdr:col>
-      <xdr:colOff>195715</xdr:colOff>
+      <xdr:col>32</xdr:col>
+      <xdr:colOff>659541</xdr:colOff>
       <xdr:row>86</xdr:row>
       <xdr:rowOff>112060</xdr:rowOff>
     </xdr:to>
@@ -10984,6 +10984,7 @@
     <col min="18" max="18" width="9.140625" customWidth="1"/>
     <col min="20" max="20" width="9.42578125" customWidth="1"/>
     <col min="22" max="22" width="10.28515625" customWidth="1"/>
+    <col min="27" max="27" width="15.85546875" customWidth="1"/>
     <col min="28" max="32" width="7.42578125" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>